<commit_message>
update euterpe insert data directus
</commit_message>
<xml_diff>
--- a/sources/euterpe/taxonomies.xlsx
+++ b/sources/euterpe/taxonomies.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rebecca\Documents\GitHub\SHERLOCK\sources\euterpe\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19F76B33-AC52-4663-8607-04253EBD5B55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7796A1C6-6F65-4812-AC79-B633CD9A6DE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="5" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11526" uniqueCount="11474">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11528" uniqueCount="11474">
   <si>
     <t>name</t>
   </si>
@@ -35305,6 +35305,9 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>11473</v>
+      </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -35443,7 +35446,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F420AD0-E833-41BC-9544-7C99816BA260}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="11.5546875" style="2"/>
@@ -35451,70 +35454,73 @@
     <col min="4" max="16384" width="11.5546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="5" customFormat="1" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:4" s="5" customFormat="1" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>11473</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>7643</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B2" s="2" t="s">
         <v>11463</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>11467</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B3" s="2" t="s">
         <v>11464</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>11468</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B4" s="2" t="s">
         <v>11465</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>11469</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B5" s="2" t="s">
         <v>11466</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>11470</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B6" s="2" t="s">
         <v>11471</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>11472</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="3"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="3"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="3"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="3"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update euterpe data insert directus (oeuvres)
</commit_message>
<xml_diff>
--- a/sources/euterpe/taxonomies.xlsx
+++ b/sources/euterpe/taxonomies.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rebecca\Documents\GitHub\SHERLOCK\sources\euterpe\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7796A1C6-6F65-4812-AC79-B633CD9A6DE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5522214-2875-4F73-8922-1BEBFBB9B4DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="5" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="spécialité" sheetId="1" r:id="rId1"/>
@@ -34534,7 +34534,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -34583,6 +34583,15 @@
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -72253,12 +72262,12 @@
   <dimension ref="A1:E495"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="28.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" style="12" customWidth="1"/>
+    <col min="1" max="1" width="12.6640625" style="21" customWidth="1"/>
     <col min="2" max="16384" width="28.44140625" style="12"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="19" t="s">
         <v>11473</v>
       </c>
       <c r="B1" s="10" t="s">
@@ -72275,7 +72284,7 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="20" t="s">
         <v>6712</v>
       </c>
       <c r="B2" s="12" t="s">
@@ -72286,7 +72295,7 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="20" t="s">
         <v>6714</v>
       </c>
       <c r="B3" s="12" t="s">
@@ -72297,7 +72306,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="20" t="s">
         <v>6716</v>
       </c>
       <c r="B4" s="12" t="s">
@@ -72308,7 +72317,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="20" t="s">
         <v>6718</v>
       </c>
       <c r="B5" s="12" t="s">
@@ -72319,7 +72328,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="20" t="s">
         <v>6720</v>
       </c>
       <c r="B6" s="12" t="s">
@@ -72330,7 +72339,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="20" t="s">
         <v>6722</v>
       </c>
       <c r="B7" s="12" t="s">
@@ -72341,7 +72350,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="20" t="s">
         <v>6724</v>
       </c>
       <c r="B8" s="12" t="s">
@@ -72352,7 +72361,7 @@
       </c>
     </row>
     <row r="9" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="20" t="s">
         <v>6726</v>
       </c>
       <c r="B9" s="12" t="s">
@@ -72363,7 +72372,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="20" t="s">
         <v>6728</v>
       </c>
       <c r="B10" s="12" t="s">
@@ -72374,7 +72383,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="20" t="s">
         <v>6730</v>
       </c>
       <c r="B11" s="12" t="s">
@@ -72385,7 +72394,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="20" t="s">
         <v>6732</v>
       </c>
       <c r="B12" s="12" t="s">
@@ -72396,7 +72405,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="20" t="s">
         <v>6734</v>
       </c>
       <c r="B13" s="12" t="s">
@@ -72407,7 +72416,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="20" t="s">
         <v>6736</v>
       </c>
       <c r="B14" s="12" t="s">
@@ -72418,7 +72427,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="20" t="s">
         <v>6738</v>
       </c>
       <c r="B15" s="12" t="s">
@@ -72429,7 +72438,7 @@
       </c>
     </row>
     <row r="16" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="20" t="s">
         <v>6740</v>
       </c>
       <c r="B16" s="12" t="s">
@@ -72440,7 +72449,7 @@
       </c>
     </row>
     <row r="17" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A17" s="11" t="s">
+      <c r="A17" s="20" t="s">
         <v>6742</v>
       </c>
       <c r="B17" s="12" t="s">
@@ -72451,7 +72460,7 @@
       </c>
     </row>
     <row r="18" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="20" t="s">
         <v>6744</v>
       </c>
       <c r="B18" s="12" t="s">
@@ -72462,7 +72471,7 @@
       </c>
     </row>
     <row r="19" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A19" s="11" t="s">
+      <c r="A19" s="20" t="s">
         <v>6746</v>
       </c>
       <c r="B19" s="12" t="s">
@@ -72473,7 +72482,7 @@
       </c>
     </row>
     <row r="20" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="20" t="s">
         <v>6748</v>
       </c>
       <c r="B20" s="12" t="s">
@@ -72484,7 +72493,7 @@
       </c>
     </row>
     <row r="21" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A21" s="11" t="s">
+      <c r="A21" s="20" t="s">
         <v>6750</v>
       </c>
       <c r="B21" s="12" t="s">
@@ -72495,7 +72504,7 @@
       </c>
     </row>
     <row r="22" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A22" s="11" t="s">
+      <c r="A22" s="20" t="s">
         <v>6752</v>
       </c>
       <c r="B22" s="12" t="s">
@@ -72506,7 +72515,7 @@
       </c>
     </row>
     <row r="23" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A23" s="11" t="s">
+      <c r="A23" s="20" t="s">
         <v>6754</v>
       </c>
       <c r="B23" s="12" t="s">
@@ -72517,7 +72526,7 @@
       </c>
     </row>
     <row r="24" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A24" s="11" t="s">
+      <c r="A24" s="20" t="s">
         <v>6756</v>
       </c>
       <c r="B24" s="12" t="s">
@@ -72528,7 +72537,7 @@
       </c>
     </row>
     <row r="25" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A25" s="11" t="s">
+      <c r="A25" s="20" t="s">
         <v>6758</v>
       </c>
       <c r="B25" s="12" t="s">
@@ -72539,7 +72548,7 @@
       </c>
     </row>
     <row r="26" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A26" s="11" t="s">
+      <c r="A26" s="20" t="s">
         <v>6760</v>
       </c>
       <c r="B26" s="12" t="s">
@@ -72550,7 +72559,7 @@
       </c>
     </row>
     <row r="27" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A27" s="11" t="s">
+      <c r="A27" s="20" t="s">
         <v>6762</v>
       </c>
       <c r="B27" s="12" t="s">
@@ -72561,7 +72570,7 @@
       </c>
     </row>
     <row r="28" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A28" s="11" t="s">
+      <c r="A28" s="20" t="s">
         <v>6764</v>
       </c>
       <c r="B28" s="12" t="s">
@@ -72572,7 +72581,7 @@
       </c>
     </row>
     <row r="29" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A29" s="11" t="s">
+      <c r="A29" s="20" t="s">
         <v>6766</v>
       </c>
       <c r="B29" s="12" t="s">
@@ -72583,7 +72592,7 @@
       </c>
     </row>
     <row r="30" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A30" s="11" t="s">
+      <c r="A30" s="20" t="s">
         <v>6768</v>
       </c>
       <c r="B30" s="12" t="s">
@@ -72594,7 +72603,7 @@
       </c>
     </row>
     <row r="31" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A31" s="11" t="s">
+      <c r="A31" s="20" t="s">
         <v>6770</v>
       </c>
       <c r="B31" s="12" t="s">
@@ -72605,7 +72614,7 @@
       </c>
     </row>
     <row r="32" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A32" s="11" t="s">
+      <c r="A32" s="20" t="s">
         <v>6772</v>
       </c>
       <c r="B32" s="12" t="s">
@@ -72616,7 +72625,7 @@
       </c>
     </row>
     <row r="33" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A33" s="11" t="s">
+      <c r="A33" s="20" t="s">
         <v>6774</v>
       </c>
       <c r="B33" s="12" t="s">
@@ -72627,7 +72636,7 @@
       </c>
     </row>
     <row r="34" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A34" s="11" t="s">
+      <c r="A34" s="20" t="s">
         <v>6776</v>
       </c>
       <c r="B34" s="12" t="s">
@@ -72638,7 +72647,7 @@
       </c>
     </row>
     <row r="35" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A35" s="11" t="s">
+      <c r="A35" s="20" t="s">
         <v>6778</v>
       </c>
       <c r="B35" s="12" t="s">
@@ -72649,7 +72658,7 @@
       </c>
     </row>
     <row r="36" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A36" s="11" t="s">
+      <c r="A36" s="20" t="s">
         <v>6780</v>
       </c>
       <c r="B36" s="12" t="s">
@@ -72660,7 +72669,7 @@
       </c>
     </row>
     <row r="37" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A37" s="11" t="s">
+      <c r="A37" s="20" t="s">
         <v>6782</v>
       </c>
       <c r="B37" s="12" t="s">
@@ -72671,7 +72680,7 @@
       </c>
     </row>
     <row r="38" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A38" s="11" t="s">
+      <c r="A38" s="20" t="s">
         <v>6784</v>
       </c>
       <c r="B38" s="12" t="s">
@@ -72682,7 +72691,7 @@
       </c>
     </row>
     <row r="39" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A39" s="11" t="s">
+      <c r="A39" s="20" t="s">
         <v>6786</v>
       </c>
       <c r="B39" s="12" t="s">
@@ -72693,7 +72702,7 @@
       </c>
     </row>
     <row r="40" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A40" s="11" t="s">
+      <c r="A40" s="20" t="s">
         <v>6788</v>
       </c>
       <c r="B40" s="12" t="s">
@@ -72704,7 +72713,7 @@
       </c>
     </row>
     <row r="41" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A41" s="11" t="s">
+      <c r="A41" s="20" t="s">
         <v>6790</v>
       </c>
       <c r="B41" s="12" t="s">
@@ -72715,7 +72724,7 @@
       </c>
     </row>
     <row r="42" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A42" s="11" t="s">
+      <c r="A42" s="20" t="s">
         <v>6792</v>
       </c>
       <c r="B42" s="12" t="s">
@@ -72726,7 +72735,7 @@
       </c>
     </row>
     <row r="43" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A43" s="11" t="s">
+      <c r="A43" s="20" t="s">
         <v>6794</v>
       </c>
       <c r="B43" s="12" t="s">
@@ -72737,7 +72746,7 @@
       </c>
     </row>
     <row r="44" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A44" s="11" t="s">
+      <c r="A44" s="20" t="s">
         <v>6796</v>
       </c>
       <c r="B44" s="12" t="s">
@@ -72748,7 +72757,7 @@
       </c>
     </row>
     <row r="45" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A45" s="11" t="s">
+      <c r="A45" s="20" t="s">
         <v>6798</v>
       </c>
       <c r="B45" s="12" t="s">
@@ -72759,7 +72768,7 @@
       </c>
     </row>
     <row r="46" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A46" s="11" t="s">
+      <c r="A46" s="20" t="s">
         <v>6800</v>
       </c>
       <c r="B46" s="12" t="s">
@@ -72770,7 +72779,7 @@
       </c>
     </row>
     <row r="47" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A47" s="11" t="s">
+      <c r="A47" s="20" t="s">
         <v>6802</v>
       </c>
       <c r="B47" s="12" t="s">
@@ -72781,7 +72790,7 @@
       </c>
     </row>
     <row r="48" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A48" s="11" t="s">
+      <c r="A48" s="20" t="s">
         <v>6804</v>
       </c>
       <c r="B48" s="12" t="s">
@@ -72792,7 +72801,7 @@
       </c>
     </row>
     <row r="49" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A49" s="11" t="s">
+      <c r="A49" s="20" t="s">
         <v>6806</v>
       </c>
       <c r="B49" s="12" t="s">
@@ -72803,7 +72812,7 @@
       </c>
     </row>
     <row r="50" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A50" s="11" t="s">
+      <c r="A50" s="20" t="s">
         <v>6808</v>
       </c>
       <c r="B50" s="12" t="s">
@@ -72814,7 +72823,7 @@
       </c>
     </row>
     <row r="51" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A51" s="11" t="s">
+      <c r="A51" s="20" t="s">
         <v>6810</v>
       </c>
       <c r="B51" s="12" t="s">
@@ -72825,7 +72834,7 @@
       </c>
     </row>
     <row r="52" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A52" s="11" t="s">
+      <c r="A52" s="20" t="s">
         <v>6812</v>
       </c>
       <c r="B52" s="12" t="s">
@@ -72836,7 +72845,7 @@
       </c>
     </row>
     <row r="53" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A53" s="11" t="s">
+      <c r="A53" s="20" t="s">
         <v>6814</v>
       </c>
       <c r="B53" s="12" t="s">
@@ -72847,7 +72856,7 @@
       </c>
     </row>
     <row r="54" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A54" s="11" t="s">
+      <c r="A54" s="20" t="s">
         <v>6816</v>
       </c>
       <c r="B54" s="12" t="s">
@@ -72858,7 +72867,7 @@
       </c>
     </row>
     <row r="55" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A55" s="11" t="s">
+      <c r="A55" s="20" t="s">
         <v>6818</v>
       </c>
       <c r="B55" s="12" t="s">
@@ -72869,7 +72878,7 @@
       </c>
     </row>
     <row r="56" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A56" s="11" t="s">
+      <c r="A56" s="20" t="s">
         <v>6820</v>
       </c>
       <c r="B56" s="12" t="s">
@@ -72880,7 +72889,7 @@
       </c>
     </row>
     <row r="57" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A57" s="11" t="s">
+      <c r="A57" s="20" t="s">
         <v>6822</v>
       </c>
       <c r="B57" s="12" t="s">
@@ -72891,7 +72900,7 @@
       </c>
     </row>
     <row r="58" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A58" s="11" t="s">
+      <c r="A58" s="20" t="s">
         <v>6824</v>
       </c>
       <c r="B58" s="12" t="s">
@@ -72902,7 +72911,7 @@
       </c>
     </row>
     <row r="59" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A59" s="11" t="s">
+      <c r="A59" s="20" t="s">
         <v>6826</v>
       </c>
       <c r="B59" s="12" t="s">
@@ -72913,7 +72922,7 @@
       </c>
     </row>
     <row r="60" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A60" s="11" t="s">
+      <c r="A60" s="20" t="s">
         <v>6828</v>
       </c>
       <c r="B60" s="12" t="s">
@@ -72924,7 +72933,7 @@
       </c>
     </row>
     <row r="61" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A61" s="11" t="s">
+      <c r="A61" s="20" t="s">
         <v>6830</v>
       </c>
       <c r="B61" s="12" t="s">
@@ -72935,7 +72944,7 @@
       </c>
     </row>
     <row r="62" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A62" s="11" t="s">
+      <c r="A62" s="20" t="s">
         <v>6832</v>
       </c>
       <c r="B62" s="12" t="s">
@@ -72946,7 +72955,7 @@
       </c>
     </row>
     <row r="63" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A63" s="11" t="s">
+      <c r="A63" s="20" t="s">
         <v>6834</v>
       </c>
       <c r="B63" s="12" t="s">
@@ -72957,7 +72966,7 @@
       </c>
     </row>
     <row r="64" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A64" s="11" t="s">
+      <c r="A64" s="20" t="s">
         <v>6836</v>
       </c>
       <c r="B64" s="12" t="s">
@@ -72968,7 +72977,7 @@
       </c>
     </row>
     <row r="65" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A65" s="11" t="s">
+      <c r="A65" s="20" t="s">
         <v>6838</v>
       </c>
       <c r="B65" s="12" t="s">
@@ -72979,7 +72988,7 @@
       </c>
     </row>
     <row r="66" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A66" s="11" t="s">
+      <c r="A66" s="20" t="s">
         <v>6840</v>
       </c>
       <c r="B66" s="12" t="s">
@@ -72990,7 +72999,7 @@
       </c>
     </row>
     <row r="67" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A67" s="11" t="s">
+      <c r="A67" s="20" t="s">
         <v>6842</v>
       </c>
       <c r="B67" s="12" t="s">
@@ -73001,7 +73010,7 @@
       </c>
     </row>
     <row r="68" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A68" s="11" t="s">
+      <c r="A68" s="20" t="s">
         <v>6844</v>
       </c>
       <c r="B68" s="12" t="s">
@@ -73012,7 +73021,7 @@
       </c>
     </row>
     <row r="69" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A69" s="11" t="s">
+      <c r="A69" s="20" t="s">
         <v>6846</v>
       </c>
       <c r="B69" s="12" t="s">
@@ -73023,7 +73032,7 @@
       </c>
     </row>
     <row r="70" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A70" s="11" t="s">
+      <c r="A70" s="20" t="s">
         <v>6848</v>
       </c>
       <c r="B70" s="12" t="s">
@@ -73034,7 +73043,7 @@
       </c>
     </row>
     <row r="71" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A71" s="11" t="s">
+      <c r="A71" s="20" t="s">
         <v>6850</v>
       </c>
       <c r="B71" s="12" t="s">
@@ -73045,7 +73054,7 @@
       </c>
     </row>
     <row r="72" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A72" s="11" t="s">
+      <c r="A72" s="20" t="s">
         <v>6852</v>
       </c>
       <c r="B72" s="12" t="s">
@@ -73056,7 +73065,7 @@
       </c>
     </row>
     <row r="73" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A73" s="11" t="s">
+      <c r="A73" s="20" t="s">
         <v>6854</v>
       </c>
       <c r="B73" s="12" t="s">
@@ -73067,7 +73076,7 @@
       </c>
     </row>
     <row r="74" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A74" s="11" t="s">
+      <c r="A74" s="20" t="s">
         <v>6856</v>
       </c>
       <c r="B74" s="12" t="s">
@@ -73078,7 +73087,7 @@
       </c>
     </row>
     <row r="75" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A75" s="11" t="s">
+      <c r="A75" s="20" t="s">
         <v>6858</v>
       </c>
       <c r="B75" s="12" t="s">
@@ -73089,7 +73098,7 @@
       </c>
     </row>
     <row r="76" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A76" s="11" t="s">
+      <c r="A76" s="20" t="s">
         <v>6860</v>
       </c>
       <c r="B76" s="12" t="s">
@@ -73100,7 +73109,7 @@
       </c>
     </row>
     <row r="77" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A77" s="11" t="s">
+      <c r="A77" s="20" t="s">
         <v>6862</v>
       </c>
       <c r="B77" s="12" t="s">
@@ -73111,7 +73120,7 @@
       </c>
     </row>
     <row r="78" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A78" s="11" t="s">
+      <c r="A78" s="20" t="s">
         <v>6864</v>
       </c>
       <c r="B78" s="12" t="s">
@@ -73122,7 +73131,7 @@
       </c>
     </row>
     <row r="79" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A79" s="11" t="s">
+      <c r="A79" s="20" t="s">
         <v>6866</v>
       </c>
       <c r="B79" s="12" t="s">
@@ -73133,7 +73142,7 @@
       </c>
     </row>
     <row r="80" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A80" s="11" t="s">
+      <c r="A80" s="20" t="s">
         <v>6868</v>
       </c>
       <c r="B80" s="12" t="s">
@@ -73144,7 +73153,7 @@
       </c>
     </row>
     <row r="81" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A81" s="11" t="s">
+      <c r="A81" s="20" t="s">
         <v>6870</v>
       </c>
       <c r="B81" s="12" t="s">
@@ -73155,7 +73164,7 @@
       </c>
     </row>
     <row r="82" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A82" s="11" t="s">
+      <c r="A82" s="20" t="s">
         <v>6872</v>
       </c>
       <c r="B82" s="12" t="s">
@@ -73166,7 +73175,7 @@
       </c>
     </row>
     <row r="83" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A83" s="11" t="s">
+      <c r="A83" s="20" t="s">
         <v>6874</v>
       </c>
       <c r="B83" s="12" t="s">
@@ -73177,7 +73186,7 @@
       </c>
     </row>
     <row r="84" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A84" s="11" t="s">
+      <c r="A84" s="20" t="s">
         <v>6876</v>
       </c>
       <c r="B84" s="12" t="s">
@@ -73188,7 +73197,7 @@
       </c>
     </row>
     <row r="85" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A85" s="11" t="s">
+      <c r="A85" s="20" t="s">
         <v>6878</v>
       </c>
       <c r="B85" s="12" t="s">
@@ -73199,7 +73208,7 @@
       </c>
     </row>
     <row r="86" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A86" s="11" t="s">
+      <c r="A86" s="20" t="s">
         <v>6880</v>
       </c>
       <c r="B86" s="12" t="s">
@@ -73210,7 +73219,7 @@
       </c>
     </row>
     <row r="87" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A87" s="11" t="s">
+      <c r="A87" s="20" t="s">
         <v>6882</v>
       </c>
       <c r="B87" s="12" t="s">
@@ -73221,7 +73230,7 @@
       </c>
     </row>
     <row r="88" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A88" s="11" t="s">
+      <c r="A88" s="20" t="s">
         <v>6884</v>
       </c>
       <c r="B88" s="12" t="s">
@@ -73232,7 +73241,7 @@
       </c>
     </row>
     <row r="89" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A89" s="11" t="s">
+      <c r="A89" s="20" t="s">
         <v>6886</v>
       </c>
       <c r="B89" s="12" t="s">
@@ -73243,7 +73252,7 @@
       </c>
     </row>
     <row r="90" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A90" s="11" t="s">
+      <c r="A90" s="20" t="s">
         <v>6888</v>
       </c>
       <c r="B90" s="12" t="s">
@@ -73254,7 +73263,7 @@
       </c>
     </row>
     <row r="91" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A91" s="11" t="s">
+      <c r="A91" s="20" t="s">
         <v>6890</v>
       </c>
       <c r="B91" s="12" t="s">
@@ -73265,7 +73274,7 @@
       </c>
     </row>
     <row r="92" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A92" s="11" t="s">
+      <c r="A92" s="20" t="s">
         <v>6892</v>
       </c>
       <c r="B92" s="12" t="s">
@@ -73276,7 +73285,7 @@
       </c>
     </row>
     <row r="93" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A93" s="11" t="s">
+      <c r="A93" s="20" t="s">
         <v>6894</v>
       </c>
       <c r="B93" s="12" t="s">
@@ -73287,7 +73296,7 @@
       </c>
     </row>
     <row r="94" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A94" s="11" t="s">
+      <c r="A94" s="20" t="s">
         <v>6896</v>
       </c>
       <c r="B94" s="12" t="s">
@@ -73298,7 +73307,7 @@
       </c>
     </row>
     <row r="95" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A95" s="11" t="s">
+      <c r="A95" s="20" t="s">
         <v>6898</v>
       </c>
       <c r="B95" s="12" t="s">
@@ -73309,7 +73318,7 @@
       </c>
     </row>
     <row r="96" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A96" s="11" t="s">
+      <c r="A96" s="20" t="s">
         <v>6900</v>
       </c>
       <c r="B96" s="12" t="s">
@@ -73320,7 +73329,7 @@
       </c>
     </row>
     <row r="97" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A97" s="11" t="s">
+      <c r="A97" s="20" t="s">
         <v>6902</v>
       </c>
       <c r="B97" s="12" t="s">
@@ -73331,7 +73340,7 @@
       </c>
     </row>
     <row r="98" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A98" s="11" t="s">
+      <c r="A98" s="20" t="s">
         <v>6904</v>
       </c>
       <c r="B98" s="12" t="s">
@@ -73342,7 +73351,7 @@
       </c>
     </row>
     <row r="99" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A99" s="11" t="s">
+      <c r="A99" s="20" t="s">
         <v>6906</v>
       </c>
       <c r="B99" s="12" t="s">
@@ -73353,7 +73362,7 @@
       </c>
     </row>
     <row r="100" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A100" s="11" t="s">
+      <c r="A100" s="20" t="s">
         <v>6908</v>
       </c>
       <c r="B100" s="12" t="s">
@@ -73364,7 +73373,7 @@
       </c>
     </row>
     <row r="101" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A101" s="11" t="s">
+      <c r="A101" s="20" t="s">
         <v>6910</v>
       </c>
       <c r="B101" s="12" t="s">
@@ -73375,7 +73384,7 @@
       </c>
     </row>
     <row r="102" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A102" s="11" t="s">
+      <c r="A102" s="20" t="s">
         <v>6912</v>
       </c>
       <c r="B102" s="12" t="s">
@@ -73386,7 +73395,7 @@
       </c>
     </row>
     <row r="103" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A103" s="11" t="s">
+      <c r="A103" s="20" t="s">
         <v>6914</v>
       </c>
       <c r="B103" s="12" t="s">
@@ -73397,7 +73406,7 @@
       </c>
     </row>
     <row r="104" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A104" s="11" t="s">
+      <c r="A104" s="20" t="s">
         <v>6916</v>
       </c>
       <c r="B104" s="12" t="s">
@@ -73408,7 +73417,7 @@
       </c>
     </row>
     <row r="105" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A105" s="11" t="s">
+      <c r="A105" s="20" t="s">
         <v>6918</v>
       </c>
       <c r="B105" s="12" t="s">
@@ -73419,7 +73428,7 @@
       </c>
     </row>
     <row r="106" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A106" s="11" t="s">
+      <c r="A106" s="20" t="s">
         <v>6920</v>
       </c>
       <c r="B106" s="12" t="s">
@@ -73430,7 +73439,7 @@
       </c>
     </row>
     <row r="107" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A107" s="11" t="s">
+      <c r="A107" s="20" t="s">
         <v>6922</v>
       </c>
       <c r="B107" s="12" t="s">
@@ -73441,7 +73450,7 @@
       </c>
     </row>
     <row r="108" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A108" s="11" t="s">
+      <c r="A108" s="20" t="s">
         <v>6924</v>
       </c>
       <c r="B108" s="12" t="s">
@@ -73452,7 +73461,7 @@
       </c>
     </row>
     <row r="109" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A109" s="11" t="s">
+      <c r="A109" s="20" t="s">
         <v>6926</v>
       </c>
       <c r="B109" s="12" t="s">
@@ -73463,7 +73472,7 @@
       </c>
     </row>
     <row r="110" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A110" s="11" t="s">
+      <c r="A110" s="20" t="s">
         <v>6928</v>
       </c>
       <c r="B110" s="12" t="s">
@@ -73474,7 +73483,7 @@
       </c>
     </row>
     <row r="111" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A111" s="11" t="s">
+      <c r="A111" s="20" t="s">
         <v>6930</v>
       </c>
       <c r="B111" s="12" t="s">
@@ -73485,7 +73494,7 @@
       </c>
     </row>
     <row r="112" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A112" s="11" t="s">
+      <c r="A112" s="20" t="s">
         <v>6932</v>
       </c>
       <c r="B112" s="12" t="s">
@@ -73496,7 +73505,7 @@
       </c>
     </row>
     <row r="113" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A113" s="11" t="s">
+      <c r="A113" s="20" t="s">
         <v>6934</v>
       </c>
       <c r="B113" s="12" t="s">
@@ -73507,7 +73516,7 @@
       </c>
     </row>
     <row r="114" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A114" s="11" t="s">
+      <c r="A114" s="20" t="s">
         <v>6936</v>
       </c>
       <c r="B114" s="12" t="s">
@@ -73518,7 +73527,7 @@
       </c>
     </row>
     <row r="115" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A115" s="11" t="s">
+      <c r="A115" s="20" t="s">
         <v>6938</v>
       </c>
       <c r="B115" s="12" t="s">
@@ -73529,7 +73538,7 @@
       </c>
     </row>
     <row r="116" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A116" s="11" t="s">
+      <c r="A116" s="20" t="s">
         <v>6940</v>
       </c>
       <c r="B116" s="12" t="s">
@@ -73540,7 +73549,7 @@
       </c>
     </row>
     <row r="117" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A117" s="11" t="s">
+      <c r="A117" s="20" t="s">
         <v>6942</v>
       </c>
       <c r="B117" s="12" t="s">
@@ -73551,7 +73560,7 @@
       </c>
     </row>
     <row r="118" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A118" s="11" t="s">
+      <c r="A118" s="20" t="s">
         <v>6944</v>
       </c>
       <c r="B118" s="12" t="s">
@@ -73562,7 +73571,7 @@
       </c>
     </row>
     <row r="119" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A119" s="11" t="s">
+      <c r="A119" s="20" t="s">
         <v>6946</v>
       </c>
       <c r="B119" s="12" t="s">
@@ -73573,7 +73582,7 @@
       </c>
     </row>
     <row r="120" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A120" s="11" t="s">
+      <c r="A120" s="20" t="s">
         <v>6948</v>
       </c>
       <c r="B120" s="12" t="s">
@@ -73584,7 +73593,7 @@
       </c>
     </row>
     <row r="121" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A121" s="11" t="s">
+      <c r="A121" s="20" t="s">
         <v>6950</v>
       </c>
       <c r="B121" s="12" t="s">
@@ -73595,7 +73604,7 @@
       </c>
     </row>
     <row r="122" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A122" s="11" t="s">
+      <c r="A122" s="20" t="s">
         <v>6952</v>
       </c>
       <c r="B122" s="12" t="s">
@@ -73606,7 +73615,7 @@
       </c>
     </row>
     <row r="123" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A123" s="11" t="s">
+      <c r="A123" s="20" t="s">
         <v>6954</v>
       </c>
       <c r="B123" s="12" t="s">
@@ -73617,7 +73626,7 @@
       </c>
     </row>
     <row r="124" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A124" s="11" t="s">
+      <c r="A124" s="20" t="s">
         <v>6956</v>
       </c>
       <c r="B124" s="12" t="s">
@@ -73628,7 +73637,7 @@
       </c>
     </row>
     <row r="125" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A125" s="11" t="s">
+      <c r="A125" s="20" t="s">
         <v>6958</v>
       </c>
       <c r="B125" s="12" t="s">
@@ -73639,7 +73648,7 @@
       </c>
     </row>
     <row r="126" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A126" s="11" t="s">
+      <c r="A126" s="20" t="s">
         <v>6960</v>
       </c>
       <c r="B126" s="12" t="s">
@@ -73650,7 +73659,7 @@
       </c>
     </row>
     <row r="127" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A127" s="11" t="s">
+      <c r="A127" s="20" t="s">
         <v>6962</v>
       </c>
       <c r="B127" s="12" t="s">
@@ -73661,7 +73670,7 @@
       </c>
     </row>
     <row r="128" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A128" s="11" t="s">
+      <c r="A128" s="20" t="s">
         <v>6964</v>
       </c>
       <c r="B128" s="12" t="s">
@@ -73672,7 +73681,7 @@
       </c>
     </row>
     <row r="129" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A129" s="11" t="s">
+      <c r="A129" s="20" t="s">
         <v>6966</v>
       </c>
       <c r="B129" s="12" t="s">
@@ -73683,7 +73692,7 @@
       </c>
     </row>
     <row r="130" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A130" s="11" t="s">
+      <c r="A130" s="20" t="s">
         <v>6968</v>
       </c>
       <c r="B130" s="12" t="s">
@@ -73694,7 +73703,7 @@
       </c>
     </row>
     <row r="131" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A131" s="11" t="s">
+      <c r="A131" s="20" t="s">
         <v>6970</v>
       </c>
       <c r="B131" s="12" t="s">
@@ -73705,7 +73714,7 @@
       </c>
     </row>
     <row r="132" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A132" s="11" t="s">
+      <c r="A132" s="20" t="s">
         <v>6972</v>
       </c>
       <c r="B132" s="12" t="s">
@@ -73716,7 +73725,7 @@
       </c>
     </row>
     <row r="133" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A133" s="11" t="s">
+      <c r="A133" s="20" t="s">
         <v>6974</v>
       </c>
       <c r="B133" s="12" t="s">
@@ -73727,7 +73736,7 @@
       </c>
     </row>
     <row r="134" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A134" s="11" t="s">
+      <c r="A134" s="20" t="s">
         <v>6976</v>
       </c>
       <c r="B134" s="12" t="s">
@@ -73738,7 +73747,7 @@
       </c>
     </row>
     <row r="135" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A135" s="11" t="s">
+      <c r="A135" s="20" t="s">
         <v>6978</v>
       </c>
       <c r="B135" s="12" t="s">
@@ -73749,7 +73758,7 @@
       </c>
     </row>
     <row r="136" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A136" s="11" t="s">
+      <c r="A136" s="20" t="s">
         <v>6980</v>
       </c>
       <c r="B136" s="12" t="s">
@@ -73760,7 +73769,7 @@
       </c>
     </row>
     <row r="137" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A137" s="11" t="s">
+      <c r="A137" s="20" t="s">
         <v>6982</v>
       </c>
       <c r="B137" s="12" t="s">
@@ -73771,7 +73780,7 @@
       </c>
     </row>
     <row r="138" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A138" s="11" t="s">
+      <c r="A138" s="20" t="s">
         <v>6984</v>
       </c>
       <c r="B138" s="12" t="s">
@@ -73782,7 +73791,7 @@
       </c>
     </row>
     <row r="139" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A139" s="11" t="s">
+      <c r="A139" s="20" t="s">
         <v>6986</v>
       </c>
       <c r="B139" s="12" t="s">
@@ -73793,7 +73802,7 @@
       </c>
     </row>
     <row r="140" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A140" s="11" t="s">
+      <c r="A140" s="20" t="s">
         <v>6988</v>
       </c>
       <c r="B140" s="12" t="s">
@@ -73804,7 +73813,7 @@
       </c>
     </row>
     <row r="141" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A141" s="11" t="s">
+      <c r="A141" s="20" t="s">
         <v>6990</v>
       </c>
       <c r="B141" s="12" t="s">
@@ -73815,7 +73824,7 @@
       </c>
     </row>
     <row r="142" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A142" s="11" t="s">
+      <c r="A142" s="20" t="s">
         <v>6992</v>
       </c>
       <c r="B142" s="12" t="s">
@@ -73826,7 +73835,7 @@
       </c>
     </row>
     <row r="143" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A143" s="11" t="s">
+      <c r="A143" s="20" t="s">
         <v>6994</v>
       </c>
       <c r="B143" s="12" t="s">
@@ -73837,7 +73846,7 @@
       </c>
     </row>
     <row r="144" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A144" s="11" t="s">
+      <c r="A144" s="20" t="s">
         <v>6996</v>
       </c>
       <c r="B144" s="12" t="s">
@@ -73848,7 +73857,7 @@
       </c>
     </row>
     <row r="145" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A145" s="11" t="s">
+      <c r="A145" s="20" t="s">
         <v>6998</v>
       </c>
       <c r="B145" s="12" t="s">
@@ -73859,7 +73868,7 @@
       </c>
     </row>
     <row r="146" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A146" s="11" t="s">
+      <c r="A146" s="20" t="s">
         <v>7000</v>
       </c>
       <c r="B146" s="12" t="s">
@@ -73870,7 +73879,7 @@
       </c>
     </row>
     <row r="147" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A147" s="11" t="s">
+      <c r="A147" s="20" t="s">
         <v>7002</v>
       </c>
       <c r="B147" s="12" t="s">
@@ -73881,7 +73890,7 @@
       </c>
     </row>
     <row r="148" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A148" s="11" t="s">
+      <c r="A148" s="20" t="s">
         <v>7004</v>
       </c>
       <c r="B148" s="12" t="s">
@@ -73892,7 +73901,7 @@
       </c>
     </row>
     <row r="149" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A149" s="11" t="s">
+      <c r="A149" s="20" t="s">
         <v>7006</v>
       </c>
       <c r="B149" s="12" t="s">
@@ -73903,7 +73912,7 @@
       </c>
     </row>
     <row r="150" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A150" s="11" t="s">
+      <c r="A150" s="20" t="s">
         <v>7008</v>
       </c>
       <c r="B150" s="12" t="s">
@@ -73914,7 +73923,7 @@
       </c>
     </row>
     <row r="151" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A151" s="11" t="s">
+      <c r="A151" s="20" t="s">
         <v>7010</v>
       </c>
       <c r="B151" s="12" t="s">
@@ -73925,7 +73934,7 @@
       </c>
     </row>
     <row r="152" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A152" s="11" t="s">
+      <c r="A152" s="20" t="s">
         <v>7012</v>
       </c>
       <c r="B152" s="12" t="s">
@@ -73936,7 +73945,7 @@
       </c>
     </row>
     <row r="153" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A153" s="11" t="s">
+      <c r="A153" s="20" t="s">
         <v>7014</v>
       </c>
       <c r="B153" s="12" t="s">
@@ -73947,7 +73956,7 @@
       </c>
     </row>
     <row r="154" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A154" s="11" t="s">
+      <c r="A154" s="20" t="s">
         <v>7016</v>
       </c>
       <c r="B154" s="12" t="s">
@@ -73958,7 +73967,7 @@
       </c>
     </row>
     <row r="155" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A155" s="11" t="s">
+      <c r="A155" s="20" t="s">
         <v>7018</v>
       </c>
       <c r="B155" s="12" t="s">
@@ -73969,7 +73978,7 @@
       </c>
     </row>
     <row r="156" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A156" s="11" t="s">
+      <c r="A156" s="20" t="s">
         <v>7020</v>
       </c>
       <c r="B156" s="12" t="s">
@@ -73980,7 +73989,7 @@
       </c>
     </row>
     <row r="157" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A157" s="11" t="s">
+      <c r="A157" s="20" t="s">
         <v>7022</v>
       </c>
       <c r="B157" s="12" t="s">
@@ -73991,7 +74000,7 @@
       </c>
     </row>
     <row r="158" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A158" s="11" t="s">
+      <c r="A158" s="20" t="s">
         <v>7024</v>
       </c>
       <c r="B158" s="12" t="s">
@@ -74002,7 +74011,7 @@
       </c>
     </row>
     <row r="159" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A159" s="11" t="s">
+      <c r="A159" s="20" t="s">
         <v>7026</v>
       </c>
       <c r="B159" s="12" t="s">
@@ -74013,7 +74022,7 @@
       </c>
     </row>
     <row r="160" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A160" s="11" t="s">
+      <c r="A160" s="20" t="s">
         <v>7028</v>
       </c>
       <c r="B160" s="12" t="s">
@@ -74024,7 +74033,7 @@
       </c>
     </row>
     <row r="161" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A161" s="11" t="s">
+      <c r="A161" s="20" t="s">
         <v>7030</v>
       </c>
       <c r="B161" s="12" t="s">
@@ -74035,7 +74044,7 @@
       </c>
     </row>
     <row r="162" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A162" s="11" t="s">
+      <c r="A162" s="20" t="s">
         <v>7032</v>
       </c>
       <c r="B162" s="12" t="s">
@@ -74046,7 +74055,7 @@
       </c>
     </row>
     <row r="163" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A163" s="11" t="s">
+      <c r="A163" s="20" t="s">
         <v>7034</v>
       </c>
       <c r="B163" s="12" t="s">
@@ -74057,7 +74066,7 @@
       </c>
     </row>
     <row r="164" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A164" s="11" t="s">
+      <c r="A164" s="20" t="s">
         <v>7036</v>
       </c>
       <c r="B164" s="12" t="s">
@@ -74068,7 +74077,7 @@
       </c>
     </row>
     <row r="165" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A165" s="11" t="s">
+      <c r="A165" s="20" t="s">
         <v>7038</v>
       </c>
       <c r="B165" s="12" t="s">
@@ -74079,7 +74088,7 @@
       </c>
     </row>
     <row r="166" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A166" s="11" t="s">
+      <c r="A166" s="20" t="s">
         <v>7040</v>
       </c>
       <c r="B166" s="12" t="s">
@@ -74090,7 +74099,7 @@
       </c>
     </row>
     <row r="167" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A167" s="11" t="s">
+      <c r="A167" s="20" t="s">
         <v>7042</v>
       </c>
       <c r="B167" s="12" t="s">
@@ -74101,7 +74110,7 @@
       </c>
     </row>
     <row r="168" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A168" s="11" t="s">
+      <c r="A168" s="20" t="s">
         <v>7044</v>
       </c>
       <c r="B168" s="12" t="s">
@@ -74112,7 +74121,7 @@
       </c>
     </row>
     <row r="169" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A169" s="11" t="s">
+      <c r="A169" s="20" t="s">
         <v>7046</v>
       </c>
       <c r="B169" s="12" t="s">
@@ -74123,7 +74132,7 @@
       </c>
     </row>
     <row r="170" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A170" s="11" t="s">
+      <c r="A170" s="20" t="s">
         <v>7048</v>
       </c>
       <c r="B170" s="12" t="s">
@@ -74134,7 +74143,7 @@
       </c>
     </row>
     <row r="171" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A171" s="11" t="s">
+      <c r="A171" s="20" t="s">
         <v>7050</v>
       </c>
       <c r="B171" s="12" t="s">
@@ -74145,7 +74154,7 @@
       </c>
     </row>
     <row r="172" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A172" s="11" t="s">
+      <c r="A172" s="20" t="s">
         <v>7052</v>
       </c>
       <c r="B172" s="12" t="s">
@@ -74156,7 +74165,7 @@
       </c>
     </row>
     <row r="173" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A173" s="11" t="s">
+      <c r="A173" s="20" t="s">
         <v>7054</v>
       </c>
       <c r="B173" s="12" t="s">
@@ -74167,7 +74176,7 @@
       </c>
     </row>
     <row r="174" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A174" s="11" t="s">
+      <c r="A174" s="20" t="s">
         <v>7056</v>
       </c>
       <c r="B174" s="12" t="s">
@@ -74178,7 +74187,7 @@
       </c>
     </row>
     <row r="175" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A175" s="11" t="s">
+      <c r="A175" s="20" t="s">
         <v>7058</v>
       </c>
       <c r="B175" s="12" t="s">
@@ -74189,7 +74198,7 @@
       </c>
     </row>
     <row r="176" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A176" s="11" t="s">
+      <c r="A176" s="20" t="s">
         <v>7060</v>
       </c>
       <c r="B176" s="12" t="s">
@@ -74200,7 +74209,7 @@
       </c>
     </row>
     <row r="177" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A177" s="11" t="s">
+      <c r="A177" s="20" t="s">
         <v>7062</v>
       </c>
       <c r="B177" s="12" t="s">
@@ -74211,7 +74220,7 @@
       </c>
     </row>
     <row r="178" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A178" s="11" t="s">
+      <c r="A178" s="20" t="s">
         <v>7064</v>
       </c>
       <c r="B178" s="12" t="s">
@@ -74222,7 +74231,7 @@
       </c>
     </row>
     <row r="179" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A179" s="11" t="s">
+      <c r="A179" s="20" t="s">
         <v>7066</v>
       </c>
       <c r="B179" s="12" t="s">
@@ -74233,7 +74242,7 @@
       </c>
     </row>
     <row r="180" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A180" s="11" t="s">
+      <c r="A180" s="20" t="s">
         <v>7068</v>
       </c>
       <c r="B180" s="12" t="s">
@@ -74244,7 +74253,7 @@
       </c>
     </row>
     <row r="181" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A181" s="11" t="s">
+      <c r="A181" s="20" t="s">
         <v>7070</v>
       </c>
       <c r="B181" s="12" t="s">
@@ -74255,7 +74264,7 @@
       </c>
     </row>
     <row r="182" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A182" s="11" t="s">
+      <c r="A182" s="20" t="s">
         <v>7072</v>
       </c>
       <c r="B182" s="12" t="s">
@@ -74266,7 +74275,7 @@
       </c>
     </row>
     <row r="183" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A183" s="11" t="s">
+      <c r="A183" s="20" t="s">
         <v>7074</v>
       </c>
       <c r="B183" s="12" t="s">
@@ -74277,7 +74286,7 @@
       </c>
     </row>
     <row r="184" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A184" s="11" t="s">
+      <c r="A184" s="20" t="s">
         <v>7076</v>
       </c>
       <c r="B184" s="12" t="s">
@@ -74288,7 +74297,7 @@
       </c>
     </row>
     <row r="185" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A185" s="11" t="s">
+      <c r="A185" s="20" t="s">
         <v>7078</v>
       </c>
       <c r="B185" s="12" t="s">
@@ -74299,7 +74308,7 @@
       </c>
     </row>
     <row r="186" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A186" s="11" t="s">
+      <c r="A186" s="20" t="s">
         <v>7080</v>
       </c>
       <c r="B186" s="12" t="s">
@@ -74310,7 +74319,7 @@
       </c>
     </row>
     <row r="187" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A187" s="11" t="s">
+      <c r="A187" s="20" t="s">
         <v>7082</v>
       </c>
       <c r="B187" s="12" t="s">
@@ -74321,7 +74330,7 @@
       </c>
     </row>
     <row r="188" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A188" s="11" t="s">
+      <c r="A188" s="20" t="s">
         <v>7084</v>
       </c>
       <c r="B188" s="12" t="s">
@@ -74332,7 +74341,7 @@
       </c>
     </row>
     <row r="189" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A189" s="11" t="s">
+      <c r="A189" s="20" t="s">
         <v>7086</v>
       </c>
       <c r="B189" s="12" t="s">
@@ -74343,7 +74352,7 @@
       </c>
     </row>
     <row r="190" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A190" s="11" t="s">
+      <c r="A190" s="20" t="s">
         <v>7088</v>
       </c>
       <c r="B190" s="12" t="s">
@@ -74354,7 +74363,7 @@
       </c>
     </row>
     <row r="191" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A191" s="11" t="s">
+      <c r="A191" s="20" t="s">
         <v>7090</v>
       </c>
       <c r="B191" s="12" t="s">
@@ -74365,7 +74374,7 @@
       </c>
     </row>
     <row r="192" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A192" s="11" t="s">
+      <c r="A192" s="20" t="s">
         <v>7092</v>
       </c>
       <c r="B192" s="12" t="s">
@@ -74376,7 +74385,7 @@
       </c>
     </row>
     <row r="193" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A193" s="11" t="s">
+      <c r="A193" s="20" t="s">
         <v>7094</v>
       </c>
       <c r="B193" s="12" t="s">
@@ -74387,7 +74396,7 @@
       </c>
     </row>
     <row r="194" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A194" s="11" t="s">
+      <c r="A194" s="20" t="s">
         <v>7096</v>
       </c>
       <c r="B194" s="12" t="s">
@@ -74398,7 +74407,7 @@
       </c>
     </row>
     <row r="195" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A195" s="11" t="s">
+      <c r="A195" s="20" t="s">
         <v>7098</v>
       </c>
       <c r="B195" s="12" t="s">
@@ -74409,7 +74418,7 @@
       </c>
     </row>
     <row r="196" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A196" s="11" t="s">
+      <c r="A196" s="20" t="s">
         <v>7100</v>
       </c>
       <c r="B196" s="12" t="s">
@@ -74420,7 +74429,7 @@
       </c>
     </row>
     <row r="197" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A197" s="11" t="s">
+      <c r="A197" s="20" t="s">
         <v>7102</v>
       </c>
       <c r="B197" s="12" t="s">
@@ -74431,7 +74440,7 @@
       </c>
     </row>
     <row r="198" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A198" s="11" t="s">
+      <c r="A198" s="20" t="s">
         <v>7104</v>
       </c>
       <c r="B198" s="12" t="s">
@@ -74442,7 +74451,7 @@
       </c>
     </row>
     <row r="199" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A199" s="11" t="s">
+      <c r="A199" s="20" t="s">
         <v>7106</v>
       </c>
       <c r="B199" s="12" t="s">
@@ -74453,7 +74462,7 @@
       </c>
     </row>
     <row r="200" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A200" s="11" t="s">
+      <c r="A200" s="20" t="s">
         <v>7108</v>
       </c>
       <c r="B200" s="12" t="s">
@@ -74464,7 +74473,7 @@
       </c>
     </row>
     <row r="201" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A201" s="11" t="s">
+      <c r="A201" s="20" t="s">
         <v>7110</v>
       </c>
       <c r="B201" s="12" t="s">
@@ -74475,7 +74484,7 @@
       </c>
     </row>
     <row r="202" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A202" s="11" t="s">
+      <c r="A202" s="20" t="s">
         <v>7112</v>
       </c>
       <c r="B202" s="12" t="s">
@@ -74486,7 +74495,7 @@
       </c>
     </row>
     <row r="203" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A203" s="11" t="s">
+      <c r="A203" s="20" t="s">
         <v>7114</v>
       </c>
       <c r="B203" s="12" t="s">
@@ -74497,7 +74506,7 @@
       </c>
     </row>
     <row r="204" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A204" s="11" t="s">
+      <c r="A204" s="20" t="s">
         <v>7116</v>
       </c>
       <c r="B204" s="12" t="s">
@@ -74508,7 +74517,7 @@
       </c>
     </row>
     <row r="205" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A205" s="11" t="s">
+      <c r="A205" s="20" t="s">
         <v>7118</v>
       </c>
       <c r="B205" s="12" t="s">
@@ -74519,7 +74528,7 @@
       </c>
     </row>
     <row r="206" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A206" s="11" t="s">
+      <c r="A206" s="20" t="s">
         <v>7120</v>
       </c>
       <c r="B206" s="12" t="s">
@@ -74530,7 +74539,7 @@
       </c>
     </row>
     <row r="207" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A207" s="11" t="s">
+      <c r="A207" s="20" t="s">
         <v>7122</v>
       </c>
       <c r="B207" s="12" t="s">
@@ -74541,7 +74550,7 @@
       </c>
     </row>
     <row r="208" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A208" s="11" t="s">
+      <c r="A208" s="20" t="s">
         <v>7124</v>
       </c>
       <c r="B208" s="12" t="s">
@@ -74552,7 +74561,7 @@
       </c>
     </row>
     <row r="209" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A209" s="11" t="s">
+      <c r="A209" s="20" t="s">
         <v>7126</v>
       </c>
       <c r="B209" s="12" t="s">
@@ -74563,7 +74572,7 @@
       </c>
     </row>
     <row r="210" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A210" s="11" t="s">
+      <c r="A210" s="20" t="s">
         <v>7128</v>
       </c>
       <c r="B210" s="12" t="s">
@@ -74574,7 +74583,7 @@
       </c>
     </row>
     <row r="211" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A211" s="11" t="s">
+      <c r="A211" s="20" t="s">
         <v>7130</v>
       </c>
       <c r="B211" s="12" t="s">
@@ -74585,7 +74594,7 @@
       </c>
     </row>
     <row r="212" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A212" s="11" t="s">
+      <c r="A212" s="20" t="s">
         <v>7132</v>
       </c>
       <c r="B212" s="12" t="s">
@@ -74596,7 +74605,7 @@
       </c>
     </row>
     <row r="213" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A213" s="11" t="s">
+      <c r="A213" s="20" t="s">
         <v>7134</v>
       </c>
       <c r="B213" s="12" t="s">
@@ -74607,7 +74616,7 @@
       </c>
     </row>
     <row r="214" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A214" s="11" t="s">
+      <c r="A214" s="20" t="s">
         <v>7136</v>
       </c>
       <c r="B214" s="12" t="s">
@@ -74618,7 +74627,7 @@
       </c>
     </row>
     <row r="215" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A215" s="11" t="s">
+      <c r="A215" s="20" t="s">
         <v>7138</v>
       </c>
       <c r="B215" s="12" t="s">
@@ -74629,7 +74638,7 @@
       </c>
     </row>
     <row r="216" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A216" s="11" t="s">
+      <c r="A216" s="20" t="s">
         <v>7140</v>
       </c>
       <c r="B216" s="12" t="s">
@@ -74640,7 +74649,7 @@
       </c>
     </row>
     <row r="217" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A217" s="11" t="s">
+      <c r="A217" s="20" t="s">
         <v>7142</v>
       </c>
       <c r="B217" s="12" t="s">
@@ -74651,7 +74660,7 @@
       </c>
     </row>
     <row r="218" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A218" s="11" t="s">
+      <c r="A218" s="20" t="s">
         <v>7144</v>
       </c>
       <c r="B218" s="12" t="s">
@@ -74662,7 +74671,7 @@
       </c>
     </row>
     <row r="219" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A219" s="11" t="s">
+      <c r="A219" s="20" t="s">
         <v>7146</v>
       </c>
       <c r="B219" s="12" t="s">
@@ -74673,7 +74682,7 @@
       </c>
     </row>
     <row r="220" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A220" s="11" t="s">
+      <c r="A220" s="20" t="s">
         <v>7148</v>
       </c>
       <c r="B220" s="12" t="s">
@@ -74684,7 +74693,7 @@
       </c>
     </row>
     <row r="221" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A221" s="11" t="s">
+      <c r="A221" s="20" t="s">
         <v>7150</v>
       </c>
       <c r="B221" s="12" t="s">
@@ -74695,7 +74704,7 @@
       </c>
     </row>
     <row r="222" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A222" s="11" t="s">
+      <c r="A222" s="20" t="s">
         <v>7152</v>
       </c>
       <c r="B222" s="12" t="s">
@@ -74706,7 +74715,7 @@
       </c>
     </row>
     <row r="223" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A223" s="11" t="s">
+      <c r="A223" s="20" t="s">
         <v>7154</v>
       </c>
       <c r="B223" s="12" t="s">
@@ -74717,7 +74726,7 @@
       </c>
     </row>
     <row r="224" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A224" s="11" t="s">
+      <c r="A224" s="20" t="s">
         <v>7156</v>
       </c>
       <c r="B224" s="12" t="s">
@@ -74728,7 +74737,7 @@
       </c>
     </row>
     <row r="225" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A225" s="11" t="s">
+      <c r="A225" s="20" t="s">
         <v>7158</v>
       </c>
       <c r="B225" s="12" t="s">
@@ -74739,7 +74748,7 @@
       </c>
     </row>
     <row r="226" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A226" s="11" t="s">
+      <c r="A226" s="20" t="s">
         <v>7160</v>
       </c>
       <c r="B226" s="12" t="s">
@@ -74750,7 +74759,7 @@
       </c>
     </row>
     <row r="227" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A227" s="11" t="s">
+      <c r="A227" s="20" t="s">
         <v>7162</v>
       </c>
       <c r="B227" s="12" t="s">
@@ -74761,7 +74770,7 @@
       </c>
     </row>
     <row r="228" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A228" s="11" t="s">
+      <c r="A228" s="20" t="s">
         <v>7164</v>
       </c>
       <c r="B228" s="12" t="s">
@@ -74772,7 +74781,7 @@
       </c>
     </row>
     <row r="229" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A229" s="11" t="s">
+      <c r="A229" s="20" t="s">
         <v>7166</v>
       </c>
       <c r="B229" s="12" t="s">
@@ -74783,7 +74792,7 @@
       </c>
     </row>
     <row r="230" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A230" s="11" t="s">
+      <c r="A230" s="20" t="s">
         <v>7168</v>
       </c>
       <c r="B230" s="12" t="s">
@@ -74794,7 +74803,7 @@
       </c>
     </row>
     <row r="231" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A231" s="11" t="s">
+      <c r="A231" s="20" t="s">
         <v>7170</v>
       </c>
       <c r="B231" s="12" t="s">
@@ -74805,7 +74814,7 @@
       </c>
     </row>
     <row r="232" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A232" s="11" t="s">
+      <c r="A232" s="20" t="s">
         <v>7172</v>
       </c>
       <c r="B232" s="12" t="s">
@@ -74816,7 +74825,7 @@
       </c>
     </row>
     <row r="233" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A233" s="11" t="s">
+      <c r="A233" s="20" t="s">
         <v>7174</v>
       </c>
       <c r="B233" s="12" t="s">
@@ -74827,7 +74836,7 @@
       </c>
     </row>
     <row r="234" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A234" s="11" t="s">
+      <c r="A234" s="20" t="s">
         <v>7176</v>
       </c>
       <c r="B234" s="12" t="s">
@@ -74838,7 +74847,7 @@
       </c>
     </row>
     <row r="235" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A235" s="11" t="s">
+      <c r="A235" s="20" t="s">
         <v>7178</v>
       </c>
       <c r="B235" s="12" t="s">
@@ -74849,7 +74858,7 @@
       </c>
     </row>
     <row r="236" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A236" s="11" t="s">
+      <c r="A236" s="20" t="s">
         <v>7180</v>
       </c>
       <c r="B236" s="12" t="s">
@@ -74860,7 +74869,7 @@
       </c>
     </row>
     <row r="237" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A237" s="11" t="s">
+      <c r="A237" s="20" t="s">
         <v>7182</v>
       </c>
       <c r="B237" s="12" t="s">
@@ -74871,7 +74880,7 @@
       </c>
     </row>
     <row r="238" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A238" s="11" t="s">
+      <c r="A238" s="20" t="s">
         <v>7184</v>
       </c>
       <c r="B238" s="12" t="s">
@@ -74882,7 +74891,7 @@
       </c>
     </row>
     <row r="239" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A239" s="11" t="s">
+      <c r="A239" s="20" t="s">
         <v>7186</v>
       </c>
       <c r="B239" s="12" t="s">
@@ -74893,7 +74902,7 @@
       </c>
     </row>
     <row r="240" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A240" s="11" t="s">
+      <c r="A240" s="20" t="s">
         <v>7188</v>
       </c>
       <c r="B240" s="12" t="s">
@@ -74904,7 +74913,7 @@
       </c>
     </row>
     <row r="241" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A241" s="11" t="s">
+      <c r="A241" s="20" t="s">
         <v>7190</v>
       </c>
       <c r="B241" s="12" t="s">
@@ -74915,7 +74924,7 @@
       </c>
     </row>
     <row r="242" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A242" s="11" t="s">
+      <c r="A242" s="20" t="s">
         <v>7192</v>
       </c>
       <c r="B242" s="12" t="s">
@@ -74926,7 +74935,7 @@
       </c>
     </row>
     <row r="243" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A243" s="11" t="s">
+      <c r="A243" s="20" t="s">
         <v>7194</v>
       </c>
       <c r="B243" s="12" t="s">
@@ -74937,7 +74946,7 @@
       </c>
     </row>
     <row r="244" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A244" s="11" t="s">
+      <c r="A244" s="20" t="s">
         <v>7196</v>
       </c>
       <c r="B244" s="12" t="s">
@@ -74948,7 +74957,7 @@
       </c>
     </row>
     <row r="245" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A245" s="11" t="s">
+      <c r="A245" s="20" t="s">
         <v>7198</v>
       </c>
       <c r="B245" s="12" t="s">
@@ -74959,7 +74968,7 @@
       </c>
     </row>
     <row r="246" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A246" s="11" t="s">
+      <c r="A246" s="20" t="s">
         <v>7200</v>
       </c>
       <c r="B246" s="12" t="s">
@@ -74970,7 +74979,7 @@
       </c>
     </row>
     <row r="247" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A247" s="11" t="s">
+      <c r="A247" s="20" t="s">
         <v>7202</v>
       </c>
       <c r="B247" s="12" t="s">
@@ -74981,7 +74990,7 @@
       </c>
     </row>
     <row r="248" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A248" s="11" t="s">
+      <c r="A248" s="20" t="s">
         <v>7204</v>
       </c>
       <c r="B248" s="12" t="s">
@@ -74992,7 +75001,7 @@
       </c>
     </row>
     <row r="249" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A249" s="11" t="s">
+      <c r="A249" s="20" t="s">
         <v>7206</v>
       </c>
       <c r="B249" s="12" t="s">
@@ -75003,7 +75012,7 @@
       </c>
     </row>
     <row r="250" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A250" s="11" t="s">
+      <c r="A250" s="20" t="s">
         <v>7208</v>
       </c>
       <c r="B250" s="12" t="s">
@@ -75014,7 +75023,7 @@
       </c>
     </row>
     <row r="251" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A251" s="11" t="s">
+      <c r="A251" s="20" t="s">
         <v>7210</v>
       </c>
       <c r="B251" s="12" t="s">
@@ -75025,7 +75034,7 @@
       </c>
     </row>
     <row r="252" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A252" s="11" t="s">
+      <c r="A252" s="20" t="s">
         <v>7212</v>
       </c>
       <c r="B252" s="12" t="s">
@@ -75036,7 +75045,7 @@
       </c>
     </row>
     <row r="253" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A253" s="11" t="s">
+      <c r="A253" s="20" t="s">
         <v>7214</v>
       </c>
       <c r="B253" s="12" t="s">
@@ -75047,7 +75056,7 @@
       </c>
     </row>
     <row r="254" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A254" s="11" t="s">
+      <c r="A254" s="20" t="s">
         <v>7216</v>
       </c>
       <c r="B254" s="12" t="s">
@@ -75058,7 +75067,7 @@
       </c>
     </row>
     <row r="255" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A255" s="11" t="s">
+      <c r="A255" s="20" t="s">
         <v>7218</v>
       </c>
       <c r="B255" s="12" t="s">
@@ -75069,7 +75078,7 @@
       </c>
     </row>
     <row r="256" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A256" s="11" t="s">
+      <c r="A256" s="20" t="s">
         <v>7220</v>
       </c>
       <c r="B256" s="12" t="s">
@@ -75080,7 +75089,7 @@
       </c>
     </row>
     <row r="257" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A257" s="11" t="s">
+      <c r="A257" s="20" t="s">
         <v>7222</v>
       </c>
       <c r="B257" s="12" t="s">
@@ -75091,7 +75100,7 @@
       </c>
     </row>
     <row r="258" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A258" s="11" t="s">
+      <c r="A258" s="20" t="s">
         <v>7224</v>
       </c>
       <c r="B258" s="12" t="s">
@@ -75102,7 +75111,7 @@
       </c>
     </row>
     <row r="259" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A259" s="11" t="s">
+      <c r="A259" s="20" t="s">
         <v>7226</v>
       </c>
       <c r="B259" s="12" t="s">
@@ -75113,7 +75122,7 @@
       </c>
     </row>
     <row r="260" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A260" s="11" t="s">
+      <c r="A260" s="20" t="s">
         <v>7228</v>
       </c>
       <c r="B260" s="12" t="s">
@@ -75124,7 +75133,7 @@
       </c>
     </row>
     <row r="261" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A261" s="11" t="s">
+      <c r="A261" s="20" t="s">
         <v>7230</v>
       </c>
       <c r="B261" s="12" t="s">
@@ -75135,7 +75144,7 @@
       </c>
     </row>
     <row r="262" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A262" s="11" t="s">
+      <c r="A262" s="20" t="s">
         <v>7232</v>
       </c>
       <c r="B262" s="12" t="s">
@@ -75146,7 +75155,7 @@
       </c>
     </row>
     <row r="263" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A263" s="11" t="s">
+      <c r="A263" s="20" t="s">
         <v>7234</v>
       </c>
       <c r="B263" s="12" t="s">
@@ -75157,7 +75166,7 @@
       </c>
     </row>
     <row r="264" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A264" s="11" t="s">
+      <c r="A264" s="20" t="s">
         <v>7236</v>
       </c>
       <c r="B264" s="12" t="s">
@@ -75168,7 +75177,7 @@
       </c>
     </row>
     <row r="265" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A265" s="11" t="s">
+      <c r="A265" s="20" t="s">
         <v>7238</v>
       </c>
       <c r="B265" s="12" t="s">
@@ -75179,7 +75188,7 @@
       </c>
     </row>
     <row r="266" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A266" s="11" t="s">
+      <c r="A266" s="20" t="s">
         <v>7240</v>
       </c>
       <c r="B266" s="12" t="s">
@@ -75190,7 +75199,7 @@
       </c>
     </row>
     <row r="267" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A267" s="11" t="s">
+      <c r="A267" s="20" t="s">
         <v>7242</v>
       </c>
       <c r="B267" s="12" t="s">
@@ -75201,7 +75210,7 @@
       </c>
     </row>
     <row r="268" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A268" s="11" t="s">
+      <c r="A268" s="20" t="s">
         <v>7244</v>
       </c>
       <c r="B268" s="12" t="s">
@@ -75212,7 +75221,7 @@
       </c>
     </row>
     <row r="269" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A269" s="11" t="s">
+      <c r="A269" s="20" t="s">
         <v>7246</v>
       </c>
       <c r="B269" s="12" t="s">
@@ -75223,7 +75232,7 @@
       </c>
     </row>
     <row r="270" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A270" s="11" t="s">
+      <c r="A270" s="20" t="s">
         <v>7248</v>
       </c>
       <c r="B270" s="12" t="s">
@@ -75234,7 +75243,7 @@
       </c>
     </row>
     <row r="271" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A271" s="11" t="s">
+      <c r="A271" s="20" t="s">
         <v>7250</v>
       </c>
       <c r="B271" s="12" t="s">
@@ -75245,7 +75254,7 @@
       </c>
     </row>
     <row r="272" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A272" s="11" t="s">
+      <c r="A272" s="20" t="s">
         <v>7252</v>
       </c>
       <c r="B272" s="12" t="s">
@@ -75256,7 +75265,7 @@
       </c>
     </row>
     <row r="273" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A273" s="11" t="s">
+      <c r="A273" s="20" t="s">
         <v>7254</v>
       </c>
       <c r="B273" s="12" t="s">
@@ -75267,7 +75276,7 @@
       </c>
     </row>
     <row r="274" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A274" s="11" t="s">
+      <c r="A274" s="20" t="s">
         <v>7256</v>
       </c>
       <c r="B274" s="12" t="s">
@@ -75278,7 +75287,7 @@
       </c>
     </row>
     <row r="275" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A275" s="11" t="s">
+      <c r="A275" s="20" t="s">
         <v>7258</v>
       </c>
       <c r="B275" s="12" t="s">
@@ -75289,7 +75298,7 @@
       </c>
     </row>
     <row r="276" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A276" s="11" t="s">
+      <c r="A276" s="20" t="s">
         <v>7260</v>
       </c>
       <c r="B276" s="12" t="s">
@@ -75300,7 +75309,7 @@
       </c>
     </row>
     <row r="277" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A277" s="11" t="s">
+      <c r="A277" s="20" t="s">
         <v>7262</v>
       </c>
       <c r="B277" s="12" t="s">
@@ -75311,7 +75320,7 @@
       </c>
     </row>
     <row r="278" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A278" s="11" t="s">
+      <c r="A278" s="20" t="s">
         <v>7264</v>
       </c>
       <c r="B278" s="12" t="s">
@@ -75322,7 +75331,7 @@
       </c>
     </row>
     <row r="279" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A279" s="11" t="s">
+      <c r="A279" s="20" t="s">
         <v>7266</v>
       </c>
       <c r="B279" s="12" t="s">
@@ -75333,7 +75342,7 @@
       </c>
     </row>
     <row r="280" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A280" s="11" t="s">
+      <c r="A280" s="20" t="s">
         <v>7268</v>
       </c>
       <c r="B280" s="12" t="s">
@@ -75344,7 +75353,7 @@
       </c>
     </row>
     <row r="281" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A281" s="11" t="s">
+      <c r="A281" s="20" t="s">
         <v>7270</v>
       </c>
       <c r="B281" s="12" t="s">
@@ -75355,7 +75364,7 @@
       </c>
     </row>
     <row r="282" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A282" s="11" t="s">
+      <c r="A282" s="20" t="s">
         <v>7272</v>
       </c>
       <c r="B282" s="12" t="s">
@@ -75366,7 +75375,7 @@
       </c>
     </row>
     <row r="283" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A283" s="11" t="s">
+      <c r="A283" s="20" t="s">
         <v>7274</v>
       </c>
       <c r="B283" s="12" t="s">
@@ -75377,7 +75386,7 @@
       </c>
     </row>
     <row r="284" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A284" s="11" t="s">
+      <c r="A284" s="20" t="s">
         <v>7276</v>
       </c>
       <c r="B284" s="12" t="s">
@@ -75388,7 +75397,7 @@
       </c>
     </row>
     <row r="285" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A285" s="11" t="s">
+      <c r="A285" s="20" t="s">
         <v>7278</v>
       </c>
       <c r="B285" s="12" t="s">
@@ -75399,7 +75408,7 @@
       </c>
     </row>
     <row r="286" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A286" s="11" t="s">
+      <c r="A286" s="20" t="s">
         <v>7280</v>
       </c>
       <c r="B286" s="12" t="s">
@@ -75410,7 +75419,7 @@
       </c>
     </row>
     <row r="287" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A287" s="11" t="s">
+      <c r="A287" s="20" t="s">
         <v>7282</v>
       </c>
       <c r="B287" s="12" t="s">
@@ -75421,7 +75430,7 @@
       </c>
     </row>
     <row r="288" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A288" s="11" t="s">
+      <c r="A288" s="20" t="s">
         <v>7284</v>
       </c>
       <c r="B288" s="12" t="s">
@@ -75432,7 +75441,7 @@
       </c>
     </row>
     <row r="289" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A289" s="11" t="s">
+      <c r="A289" s="20" t="s">
         <v>7286</v>
       </c>
       <c r="B289" s="12" t="s">
@@ -75443,7 +75452,7 @@
       </c>
     </row>
     <row r="290" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A290" s="11" t="s">
+      <c r="A290" s="20" t="s">
         <v>7288</v>
       </c>
       <c r="B290" s="12" t="s">
@@ -75454,7 +75463,7 @@
       </c>
     </row>
     <row r="291" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A291" s="11" t="s">
+      <c r="A291" s="20" t="s">
         <v>7290</v>
       </c>
       <c r="B291" s="12" t="s">
@@ -75465,7 +75474,7 @@
       </c>
     </row>
     <row r="292" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A292" s="11" t="s">
+      <c r="A292" s="20" t="s">
         <v>7292</v>
       </c>
       <c r="B292" s="12" t="s">
@@ -75476,7 +75485,7 @@
       </c>
     </row>
     <row r="293" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A293" s="11" t="s">
+      <c r="A293" s="20" t="s">
         <v>7294</v>
       </c>
       <c r="B293" s="12" t="s">
@@ -75487,7 +75496,7 @@
       </c>
     </row>
     <row r="294" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A294" s="11" t="s">
+      <c r="A294" s="20" t="s">
         <v>7296</v>
       </c>
       <c r="B294" s="12" t="s">
@@ -75498,7 +75507,7 @@
       </c>
     </row>
     <row r="295" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A295" s="11" t="s">
+      <c r="A295" s="20" t="s">
         <v>7298</v>
       </c>
       <c r="B295" s="12" t="s">
@@ -75509,7 +75518,7 @@
       </c>
     </row>
     <row r="296" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A296" s="11" t="s">
+      <c r="A296" s="20" t="s">
         <v>7300</v>
       </c>
       <c r="B296" s="12" t="s">
@@ -75520,7 +75529,7 @@
       </c>
     </row>
     <row r="297" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A297" s="11" t="s">
+      <c r="A297" s="20" t="s">
         <v>7302</v>
       </c>
       <c r="B297" s="12" t="s">
@@ -75531,7 +75540,7 @@
       </c>
     </row>
     <row r="298" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A298" s="11" t="s">
+      <c r="A298" s="20" t="s">
         <v>7304</v>
       </c>
       <c r="B298" s="12" t="s">
@@ -75542,7 +75551,7 @@
       </c>
     </row>
     <row r="299" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A299" s="11" t="s">
+      <c r="A299" s="20" t="s">
         <v>7306</v>
       </c>
       <c r="B299" s="12" t="s">
@@ -75553,7 +75562,7 @@
       </c>
     </row>
     <row r="300" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A300" s="11" t="s">
+      <c r="A300" s="20" t="s">
         <v>7308</v>
       </c>
       <c r="B300" s="12" t="s">
@@ -75564,7 +75573,7 @@
       </c>
     </row>
     <row r="301" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A301" s="11" t="s">
+      <c r="A301" s="20" t="s">
         <v>7310</v>
       </c>
       <c r="B301" s="12" t="s">
@@ -75575,7 +75584,7 @@
       </c>
     </row>
     <row r="302" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A302" s="11" t="s">
+      <c r="A302" s="20" t="s">
         <v>7312</v>
       </c>
       <c r="B302" s="12" t="s">
@@ -75586,7 +75595,7 @@
       </c>
     </row>
     <row r="303" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A303" s="11" t="s">
+      <c r="A303" s="20" t="s">
         <v>7314</v>
       </c>
       <c r="B303" s="12" t="s">
@@ -75597,7 +75606,7 @@
       </c>
     </row>
     <row r="304" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A304" s="11" t="s">
+      <c r="A304" s="20" t="s">
         <v>7316</v>
       </c>
       <c r="B304" s="12" t="s">
@@ -75608,7 +75617,7 @@
       </c>
     </row>
     <row r="305" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A305" s="11" t="s">
+      <c r="A305" s="20" t="s">
         <v>7318</v>
       </c>
       <c r="B305" s="12" t="s">
@@ -75619,7 +75628,7 @@
       </c>
     </row>
     <row r="306" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A306" s="11" t="s">
+      <c r="A306" s="20" t="s">
         <v>7320</v>
       </c>
       <c r="B306" s="12" t="s">
@@ -75630,7 +75639,7 @@
       </c>
     </row>
     <row r="307" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A307" s="11" t="s">
+      <c r="A307" s="20" t="s">
         <v>7322</v>
       </c>
       <c r="B307" s="12" t="s">
@@ -75641,7 +75650,7 @@
       </c>
     </row>
     <row r="308" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A308" s="11" t="s">
+      <c r="A308" s="20" t="s">
         <v>7324</v>
       </c>
       <c r="B308" s="12" t="s">
@@ -75652,7 +75661,7 @@
       </c>
     </row>
     <row r="309" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A309" s="11" t="s">
+      <c r="A309" s="20" t="s">
         <v>7326</v>
       </c>
       <c r="B309" s="12" t="s">
@@ -75663,7 +75672,7 @@
       </c>
     </row>
     <row r="310" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A310" s="11" t="s">
+      <c r="A310" s="20" t="s">
         <v>7328</v>
       </c>
       <c r="B310" s="12" t="s">
@@ -75674,7 +75683,7 @@
       </c>
     </row>
     <row r="311" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A311" s="11" t="s">
+      <c r="A311" s="20" t="s">
         <v>7330</v>
       </c>
       <c r="B311" s="12" t="s">
@@ -75685,7 +75694,7 @@
       </c>
     </row>
     <row r="312" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A312" s="11" t="s">
+      <c r="A312" s="20" t="s">
         <v>7332</v>
       </c>
       <c r="B312" s="12" t="s">
@@ -75696,7 +75705,7 @@
       </c>
     </row>
     <row r="313" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A313" s="11" t="s">
+      <c r="A313" s="20" t="s">
         <v>7334</v>
       </c>
       <c r="B313" s="12" t="s">
@@ -75707,7 +75716,7 @@
       </c>
     </row>
     <row r="314" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A314" s="11" t="s">
+      <c r="A314" s="20" t="s">
         <v>7336</v>
       </c>
       <c r="B314" s="12" t="s">
@@ -75718,7 +75727,7 @@
       </c>
     </row>
     <row r="315" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A315" s="11" t="s">
+      <c r="A315" s="20" t="s">
         <v>7338</v>
       </c>
       <c r="B315" s="12" t="s">
@@ -75729,7 +75738,7 @@
       </c>
     </row>
     <row r="316" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A316" s="11" t="s">
+      <c r="A316" s="20" t="s">
         <v>7340</v>
       </c>
       <c r="B316" s="12" t="s">
@@ -75740,7 +75749,7 @@
       </c>
     </row>
     <row r="317" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A317" s="11" t="s">
+      <c r="A317" s="20" t="s">
         <v>7342</v>
       </c>
       <c r="B317" s="12" t="s">
@@ -75751,7 +75760,7 @@
       </c>
     </row>
     <row r="318" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A318" s="11" t="s">
+      <c r="A318" s="20" t="s">
         <v>7344</v>
       </c>
       <c r="B318" s="12" t="s">
@@ -75762,7 +75771,7 @@
       </c>
     </row>
     <row r="319" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A319" s="11" t="s">
+      <c r="A319" s="20" t="s">
         <v>7346</v>
       </c>
       <c r="B319" s="12" t="s">
@@ -75773,7 +75782,7 @@
       </c>
     </row>
     <row r="320" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A320" s="11" t="s">
+      <c r="A320" s="20" t="s">
         <v>7348</v>
       </c>
       <c r="B320" s="12" t="s">
@@ -75784,7 +75793,7 @@
       </c>
     </row>
     <row r="321" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A321" s="11" t="s">
+      <c r="A321" s="20" t="s">
         <v>7350</v>
       </c>
       <c r="B321" s="12" t="s">
@@ -75795,7 +75804,7 @@
       </c>
     </row>
     <row r="322" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A322" s="11" t="s">
+      <c r="A322" s="20" t="s">
         <v>7352</v>
       </c>
       <c r="B322" s="12" t="s">
@@ -75806,7 +75815,7 @@
       </c>
     </row>
     <row r="323" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A323" s="11" t="s">
+      <c r="A323" s="20" t="s">
         <v>7354</v>
       </c>
       <c r="B323" s="12" t="s">
@@ -75817,7 +75826,7 @@
       </c>
     </row>
     <row r="324" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A324" s="11" t="s">
+      <c r="A324" s="20" t="s">
         <v>7356</v>
       </c>
       <c r="B324" s="12" t="s">
@@ -75828,7 +75837,7 @@
       </c>
     </row>
     <row r="325" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A325" s="11" t="s">
+      <c r="A325" s="20" t="s">
         <v>7358</v>
       </c>
       <c r="B325" s="12" t="s">
@@ -75839,7 +75848,7 @@
       </c>
     </row>
     <row r="326" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A326" s="11" t="s">
+      <c r="A326" s="20" t="s">
         <v>7360</v>
       </c>
       <c r="B326" s="12" t="s">
@@ -75850,7 +75859,7 @@
       </c>
     </row>
     <row r="327" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A327" s="11" t="s">
+      <c r="A327" s="20" t="s">
         <v>7362</v>
       </c>
       <c r="B327" s="12" t="s">
@@ -75861,7 +75870,7 @@
       </c>
     </row>
     <row r="328" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A328" s="11" t="s">
+      <c r="A328" s="20" t="s">
         <v>7364</v>
       </c>
       <c r="B328" s="12" t="s">
@@ -75872,7 +75881,7 @@
       </c>
     </row>
     <row r="329" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A329" s="11" t="s">
+      <c r="A329" s="20" t="s">
         <v>7366</v>
       </c>
       <c r="B329" s="12" t="s">
@@ -75883,7 +75892,7 @@
       </c>
     </row>
     <row r="330" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A330" s="11" t="s">
+      <c r="A330" s="20" t="s">
         <v>7368</v>
       </c>
       <c r="B330" s="12" t="s">
@@ -75894,7 +75903,7 @@
       </c>
     </row>
     <row r="331" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A331" s="11" t="s">
+      <c r="A331" s="20" t="s">
         <v>7370</v>
       </c>
       <c r="B331" s="12" t="s">
@@ -75905,7 +75914,7 @@
       </c>
     </row>
     <row r="332" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A332" s="11" t="s">
+      <c r="A332" s="20" t="s">
         <v>7372</v>
       </c>
       <c r="B332" s="12" t="s">
@@ -75916,7 +75925,7 @@
       </c>
     </row>
     <row r="333" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A333" s="11" t="s">
+      <c r="A333" s="20" t="s">
         <v>7374</v>
       </c>
       <c r="B333" s="12" t="s">
@@ -75927,7 +75936,7 @@
       </c>
     </row>
     <row r="334" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A334" s="11" t="s">
+      <c r="A334" s="20" t="s">
         <v>7376</v>
       </c>
       <c r="B334" s="12" t="s">
@@ -75938,7 +75947,7 @@
       </c>
     </row>
     <row r="335" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A335" s="11" t="s">
+      <c r="A335" s="20" t="s">
         <v>7378</v>
       </c>
       <c r="B335" s="12" t="s">
@@ -75949,7 +75958,7 @@
       </c>
     </row>
     <row r="336" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A336" s="11" t="s">
+      <c r="A336" s="20" t="s">
         <v>7380</v>
       </c>
       <c r="B336" s="12" t="s">
@@ -75960,7 +75969,7 @@
       </c>
     </row>
     <row r="337" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A337" s="11" t="s">
+      <c r="A337" s="20" t="s">
         <v>7382</v>
       </c>
       <c r="B337" s="12" t="s">
@@ -75971,7 +75980,7 @@
       </c>
     </row>
     <row r="338" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A338" s="11" t="s">
+      <c r="A338" s="20" t="s">
         <v>7384</v>
       </c>
       <c r="B338" s="12" t="s">
@@ -75982,7 +75991,7 @@
       </c>
     </row>
     <row r="339" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A339" s="11" t="s">
+      <c r="A339" s="20" t="s">
         <v>7386</v>
       </c>
       <c r="B339" s="12" t="s">
@@ -75993,7 +76002,7 @@
       </c>
     </row>
     <row r="340" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A340" s="11" t="s">
+      <c r="A340" s="20" t="s">
         <v>7388</v>
       </c>
       <c r="B340" s="12" t="s">
@@ -76004,7 +76013,7 @@
       </c>
     </row>
     <row r="341" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A341" s="11" t="s">
+      <c r="A341" s="20" t="s">
         <v>7390</v>
       </c>
       <c r="B341" s="12" t="s">
@@ -76015,7 +76024,7 @@
       </c>
     </row>
     <row r="342" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A342" s="11" t="s">
+      <c r="A342" s="20" t="s">
         <v>7392</v>
       </c>
       <c r="B342" s="12" t="s">
@@ -76026,7 +76035,7 @@
       </c>
     </row>
     <row r="343" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A343" s="11" t="s">
+      <c r="A343" s="20" t="s">
         <v>7394</v>
       </c>
       <c r="B343" s="12" t="s">
@@ -76037,7 +76046,7 @@
       </c>
     </row>
     <row r="344" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A344" s="11" t="s">
+      <c r="A344" s="20" t="s">
         <v>7396</v>
       </c>
       <c r="B344" s="12" t="s">
@@ -76048,7 +76057,7 @@
       </c>
     </row>
     <row r="345" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A345" s="11" t="s">
+      <c r="A345" s="20" t="s">
         <v>7398</v>
       </c>
       <c r="B345" s="12" t="s">
@@ -76059,7 +76068,7 @@
       </c>
     </row>
     <row r="346" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A346" s="11" t="s">
+      <c r="A346" s="20" t="s">
         <v>7400</v>
       </c>
       <c r="B346" s="12" t="s">
@@ -76070,7 +76079,7 @@
       </c>
     </row>
     <row r="347" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A347" s="11" t="s">
+      <c r="A347" s="20" t="s">
         <v>7402</v>
       </c>
       <c r="B347" s="12" t="s">
@@ -76081,7 +76090,7 @@
       </c>
     </row>
     <row r="348" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A348" s="11" t="s">
+      <c r="A348" s="20" t="s">
         <v>7404</v>
       </c>
       <c r="B348" s="12" t="s">
@@ -76092,7 +76101,7 @@
       </c>
     </row>
     <row r="349" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A349" s="11" t="s">
+      <c r="A349" s="20" t="s">
         <v>7406</v>
       </c>
       <c r="B349" s="12" t="s">
@@ -76103,7 +76112,7 @@
       </c>
     </row>
     <row r="350" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A350" s="11" t="s">
+      <c r="A350" s="20" t="s">
         <v>7408</v>
       </c>
       <c r="B350" s="12" t="s">
@@ -76114,7 +76123,7 @@
       </c>
     </row>
     <row r="351" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A351" s="11" t="s">
+      <c r="A351" s="20" t="s">
         <v>7410</v>
       </c>
       <c r="B351" s="12" t="s">
@@ -76125,7 +76134,7 @@
       </c>
     </row>
     <row r="352" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A352" s="11" t="s">
+      <c r="A352" s="20" t="s">
         <v>7412</v>
       </c>
       <c r="B352" s="12" t="s">
@@ -76136,7 +76145,7 @@
       </c>
     </row>
     <row r="353" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A353" s="11" t="s">
+      <c r="A353" s="20" t="s">
         <v>7414</v>
       </c>
       <c r="B353" s="12" t="s">
@@ -76147,7 +76156,7 @@
       </c>
     </row>
     <row r="354" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A354" s="11" t="s">
+      <c r="A354" s="20" t="s">
         <v>7416</v>
       </c>
       <c r="B354" s="12" t="s">
@@ -76158,7 +76167,7 @@
       </c>
     </row>
     <row r="355" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A355" s="11" t="s">
+      <c r="A355" s="20" t="s">
         <v>7418</v>
       </c>
       <c r="B355" s="12" t="s">
@@ -76169,7 +76178,7 @@
       </c>
     </row>
     <row r="356" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A356" s="11" t="s">
+      <c r="A356" s="20" t="s">
         <v>7420</v>
       </c>
       <c r="B356" s="12" t="s">
@@ -76180,7 +76189,7 @@
       </c>
     </row>
     <row r="357" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A357" s="11" t="s">
+      <c r="A357" s="20" t="s">
         <v>7422</v>
       </c>
       <c r="B357" s="12" t="s">
@@ -76191,7 +76200,7 @@
       </c>
     </row>
     <row r="358" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A358" s="11" t="s">
+      <c r="A358" s="20" t="s">
         <v>7424</v>
       </c>
       <c r="B358" s="12" t="s">
@@ -76202,7 +76211,7 @@
       </c>
     </row>
     <row r="359" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A359" s="11" t="s">
+      <c r="A359" s="20" t="s">
         <v>7426</v>
       </c>
       <c r="B359" s="12" t="s">
@@ -76213,7 +76222,7 @@
       </c>
     </row>
     <row r="360" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A360" s="11" t="s">
+      <c r="A360" s="20" t="s">
         <v>7428</v>
       </c>
       <c r="B360" s="12" t="s">
@@ -76224,7 +76233,7 @@
       </c>
     </row>
     <row r="361" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A361" s="11" t="s">
+      <c r="A361" s="20" t="s">
         <v>7430</v>
       </c>
       <c r="B361" s="12" t="s">
@@ -76235,7 +76244,7 @@
       </c>
     </row>
     <row r="362" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A362" s="11" t="s">
+      <c r="A362" s="20" t="s">
         <v>7432</v>
       </c>
       <c r="B362" s="12" t="s">
@@ -76246,7 +76255,7 @@
       </c>
     </row>
     <row r="363" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A363" s="11" t="s">
+      <c r="A363" s="20" t="s">
         <v>7434</v>
       </c>
       <c r="B363" s="12" t="s">
@@ -76257,7 +76266,7 @@
       </c>
     </row>
     <row r="364" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A364" s="11" t="s">
+      <c r="A364" s="20" t="s">
         <v>7436</v>
       </c>
       <c r="B364" s="12" t="s">
@@ -76268,7 +76277,7 @@
       </c>
     </row>
     <row r="365" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A365" s="11" t="s">
+      <c r="A365" s="20" t="s">
         <v>7438</v>
       </c>
       <c r="B365" s="12" t="s">
@@ -76279,7 +76288,7 @@
       </c>
     </row>
     <row r="366" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A366" s="11" t="s">
+      <c r="A366" s="20" t="s">
         <v>7440</v>
       </c>
       <c r="B366" s="12" t="s">
@@ -76290,7 +76299,7 @@
       </c>
     </row>
     <row r="367" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A367" s="11" t="s">
+      <c r="A367" s="20" t="s">
         <v>7442</v>
       </c>
       <c r="B367" s="12" t="s">
@@ -76301,7 +76310,7 @@
       </c>
     </row>
     <row r="368" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A368" s="11" t="s">
+      <c r="A368" s="20" t="s">
         <v>7444</v>
       </c>
       <c r="B368" s="12" t="s">
@@ -76312,7 +76321,7 @@
       </c>
     </row>
     <row r="369" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A369" s="11" t="s">
+      <c r="A369" s="20" t="s">
         <v>7446</v>
       </c>
       <c r="B369" s="12" t="s">
@@ -76323,7 +76332,7 @@
       </c>
     </row>
     <row r="370" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A370" s="11" t="s">
+      <c r="A370" s="20" t="s">
         <v>7448</v>
       </c>
       <c r="B370" s="12" t="s">
@@ -76334,7 +76343,7 @@
       </c>
     </row>
     <row r="371" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A371" s="11" t="s">
+      <c r="A371" s="20" t="s">
         <v>7450</v>
       </c>
       <c r="B371" s="12" t="s">
@@ -76345,7 +76354,7 @@
       </c>
     </row>
     <row r="372" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A372" s="11" t="s">
+      <c r="A372" s="20" t="s">
         <v>7452</v>
       </c>
       <c r="B372" s="12" t="s">
@@ -76356,7 +76365,7 @@
       </c>
     </row>
     <row r="373" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A373" s="11" t="s">
+      <c r="A373" s="20" t="s">
         <v>7454</v>
       </c>
       <c r="B373" s="12" t="s">
@@ -76367,7 +76376,7 @@
       </c>
     </row>
     <row r="374" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A374" s="11" t="s">
+      <c r="A374" s="20" t="s">
         <v>7456</v>
       </c>
       <c r="B374" s="12" t="s">
@@ -76378,7 +76387,7 @@
       </c>
     </row>
     <row r="375" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A375" s="11" t="s">
+      <c r="A375" s="20" t="s">
         <v>7458</v>
       </c>
       <c r="B375" s="12" t="s">
@@ -76389,7 +76398,7 @@
       </c>
     </row>
     <row r="376" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A376" s="11" t="s">
+      <c r="A376" s="20" t="s">
         <v>7460</v>
       </c>
       <c r="B376" s="12" t="s">
@@ -76400,7 +76409,7 @@
       </c>
     </row>
     <row r="377" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A377" s="11" t="s">
+      <c r="A377" s="20" t="s">
         <v>7462</v>
       </c>
       <c r="B377" s="12" t="s">
@@ -76411,7 +76420,7 @@
       </c>
     </row>
     <row r="378" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A378" s="11" t="s">
+      <c r="A378" s="20" t="s">
         <v>7464</v>
       </c>
       <c r="B378" s="12" t="s">
@@ -76422,7 +76431,7 @@
       </c>
     </row>
     <row r="379" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A379" s="11" t="s">
+      <c r="A379" s="20" t="s">
         <v>7466</v>
       </c>
       <c r="B379" s="12" t="s">
@@ -76433,7 +76442,7 @@
       </c>
     </row>
     <row r="380" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A380" s="11" t="s">
+      <c r="A380" s="20" t="s">
         <v>7468</v>
       </c>
       <c r="B380" s="12" t="s">
@@ -76444,7 +76453,7 @@
       </c>
     </row>
     <row r="381" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A381" s="11" t="s">
+      <c r="A381" s="20" t="s">
         <v>7470</v>
       </c>
       <c r="B381" s="12" t="s">
@@ -76455,7 +76464,7 @@
       </c>
     </row>
     <row r="382" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A382" s="11" t="s">
+      <c r="A382" s="20" t="s">
         <v>7472</v>
       </c>
       <c r="B382" s="12" t="s">
@@ -76466,7 +76475,7 @@
       </c>
     </row>
     <row r="383" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A383" s="11" t="s">
+      <c r="A383" s="20" t="s">
         <v>7474</v>
       </c>
       <c r="B383" s="12" t="s">
@@ -76477,7 +76486,7 @@
       </c>
     </row>
     <row r="384" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A384" s="11" t="s">
+      <c r="A384" s="20" t="s">
         <v>7476</v>
       </c>
       <c r="B384" s="12" t="s">
@@ -76488,7 +76497,7 @@
       </c>
     </row>
     <row r="385" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A385" s="11" t="s">
+      <c r="A385" s="20" t="s">
         <v>7478</v>
       </c>
       <c r="B385" s="12" t="s">
@@ -76499,7 +76508,7 @@
       </c>
     </row>
     <row r="386" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A386" s="11" t="s">
+      <c r="A386" s="20" t="s">
         <v>7480</v>
       </c>
       <c r="B386" s="12" t="s">
@@ -76510,7 +76519,7 @@
       </c>
     </row>
     <row r="387" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A387" s="11" t="s">
+      <c r="A387" s="20" t="s">
         <v>7482</v>
       </c>
       <c r="B387" s="12" t="s">
@@ -76521,7 +76530,7 @@
       </c>
     </row>
     <row r="388" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A388" s="11" t="s">
+      <c r="A388" s="20" t="s">
         <v>7484</v>
       </c>
       <c r="B388" s="12" t="s">
@@ -76532,7 +76541,7 @@
       </c>
     </row>
     <row r="389" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A389" s="11" t="s">
+      <c r="A389" s="20" t="s">
         <v>7486</v>
       </c>
       <c r="B389" s="12" t="s">
@@ -76543,7 +76552,7 @@
       </c>
     </row>
     <row r="390" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A390" s="11" t="s">
+      <c r="A390" s="20" t="s">
         <v>7488</v>
       </c>
       <c r="B390" s="12" t="s">
@@ -76554,7 +76563,7 @@
       </c>
     </row>
     <row r="391" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A391" s="11" t="s">
+      <c r="A391" s="20" t="s">
         <v>7490</v>
       </c>
       <c r="B391" s="12" t="s">
@@ -76565,7 +76574,7 @@
       </c>
     </row>
     <row r="392" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A392" s="11" t="s">
+      <c r="A392" s="20" t="s">
         <v>7492</v>
       </c>
       <c r="B392" s="12" t="s">
@@ -76576,7 +76585,7 @@
       </c>
     </row>
     <row r="393" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A393" s="11" t="s">
+      <c r="A393" s="20" t="s">
         <v>7494</v>
       </c>
       <c r="B393" s="12" t="s">
@@ -76587,7 +76596,7 @@
       </c>
     </row>
     <row r="394" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A394" s="11" t="s">
+      <c r="A394" s="20" t="s">
         <v>7496</v>
       </c>
       <c r="B394" s="12" t="s">
@@ -76598,7 +76607,7 @@
       </c>
     </row>
     <row r="395" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A395" s="11" t="s">
+      <c r="A395" s="20" t="s">
         <v>7498</v>
       </c>
       <c r="B395" s="12" t="s">
@@ -76609,7 +76618,7 @@
       </c>
     </row>
     <row r="396" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A396" s="11" t="s">
+      <c r="A396" s="20" t="s">
         <v>7500</v>
       </c>
       <c r="B396" s="12" t="s">
@@ -76620,7 +76629,7 @@
       </c>
     </row>
     <row r="397" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A397" s="11" t="s">
+      <c r="A397" s="20" t="s">
         <v>7502</v>
       </c>
       <c r="B397" s="12" t="s">
@@ -76631,7 +76640,7 @@
       </c>
     </row>
     <row r="398" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A398" s="11" t="s">
+      <c r="A398" s="20" t="s">
         <v>7504</v>
       </c>
       <c r="B398" s="12" t="s">
@@ -76642,7 +76651,7 @@
       </c>
     </row>
     <row r="399" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A399" s="11" t="s">
+      <c r="A399" s="20" t="s">
         <v>7506</v>
       </c>
       <c r="B399" s="12" t="s">
@@ -76653,7 +76662,7 @@
       </c>
     </row>
     <row r="400" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A400" s="11" t="s">
+      <c r="A400" s="20" t="s">
         <v>7508</v>
       </c>
       <c r="B400" s="12" t="s">
@@ -76664,7 +76673,7 @@
       </c>
     </row>
     <row r="401" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A401" s="11" t="s">
+      <c r="A401" s="20" t="s">
         <v>7510</v>
       </c>
       <c r="B401" s="12" t="s">
@@ -76675,7 +76684,7 @@
       </c>
     </row>
     <row r="402" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A402" s="11" t="s">
+      <c r="A402" s="20" t="s">
         <v>7512</v>
       </c>
       <c r="B402" s="12" t="s">
@@ -76686,7 +76695,7 @@
       </c>
     </row>
     <row r="403" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A403" s="11" t="s">
+      <c r="A403" s="20" t="s">
         <v>7514</v>
       </c>
       <c r="B403" s="12" t="s">

</xml_diff>